<commit_message>
Finalize Phase 03 sequence 1-14 and remove redundant identifiers
</commit_message>
<xml_diff>
--- a/003_Geocoding_and_Validation/places_geocoded.xlsx
+++ b/003_Geocoding_and_Validation/places_geocoded.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'places'!$A$1:$Q$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'places'!$A$1:$P$15</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1114,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="15.6640625" customWidth="1" style="9" min="7" max="7"/>
@@ -1126,85 +1126,80 @@
     <row r="1" ht="34" customFormat="1" customHeight="1" s="4">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>id重新编号</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>sequence</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>sequence</t>
+          <t>gaspar_name</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>gaspar_name</t>
+          <t>modern_name</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>modern_name</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>display_level</t>
+        </is>
+      </c>
       <c r="G1" s="7" t="inlineStr">
         <is>
-          <t>display_level</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
           <t>location_precision</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>coordinate_status</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>coordinate_status</t>
+          <t>place_type</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>place_type</t>
+          <t>original_spanish</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
-          <t>original_spanish</t>
+          <t>chinese_translation</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>chinese_translation</t>
+          <t>image_url</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
         <is>
-          <t>image_url</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
-        <is>
           <t>model_3d_url</t>
         </is>
       </c>
-      <c r="Q1" s="0" t="inlineStr">
+      <c r="P1" s="0" t="inlineStr">
         <is>
           <t>coordinate_source</t>
         </is>
@@ -1213,20 +1208,20 @@
     <row r="2" ht="34" customHeight="1" s="9">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
           <t>1880-03-26</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Macao</t>
+        </is>
+      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Macao</t>
+          <t>澳门</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1234,45 +1229,45 @@
           <t>澳门</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>澳门</t>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H2" s="8" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="H2" s="2" t="n">
+        <v>22.19</v>
+      </c>
       <c r="I2" s="2" t="n">
-        <v>22.19</v>
-      </c>
-      <c r="J2" s="2" t="n">
         <v>113.538056</v>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>city-level</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>city-level</t>
+          <t>城市</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>城市</t>
+          <t>Macao, 26 de Marzo de 1880.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Macao, 26 de Marzo de 1880.</t>
+          <t>澳门，1880年3月26日。</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>澳门，1880年3月26日。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -1280,12 +1275,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q2" s="0" t="inlineStr">
+      <c r="P2" s="0" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Special:EntityData/Q14773.json</t>
         </is>
@@ -1294,79 +1284,74 @@
     <row r="3" ht="187" customHeight="1" s="9">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P004</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
           <t>1881-01-30</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>procesión de linternas</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>procesión de linternas</t>
+          <t>香港：长洲太平清醮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>香港：长洲太平清醮</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
           <t>香港</t>
         </is>
       </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="H3" s="2" t="n">
+        <v>22.278333</v>
+      </c>
       <c r="I3" s="2" t="n">
-        <v>22.278333</v>
-      </c>
-      <c r="J3" s="2" t="n">
         <v>114.158611</v>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>city-level</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>city-level</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
           <t>地方节庆</t>
         </is>
       </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Es la primera vez que he visto realizado el esplendor de mi China soñada. Desgraciadamente sólo dura la ilusión ocho días al año. Quince minutos han bastado muchas veces para que un incendio lo devorase todo...</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Es la primera vez que he visto realizado el esplendor de mi China soñada. Desgraciadamente sólo dura la ilusión ocho días al año. Quince minutos han bastado muchas veces para que un incendio lo devorase todo...</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
           <t>这是我第一次看到我梦中的中国之辉煌成为现实。不幸的是，这种幻象每年只持续八天。很多时候，十五分钟就足以让一场大火吞噬一切……</t>
         </is>
       </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
           <t>null</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q3" s="0" t="inlineStr">
+      <c r="P3" s="0" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Special:EntityData/Q8646.json</t>
         </is>
@@ -1375,66 +1360,66 @@
     <row r="4" ht="204" customFormat="1" customHeight="1" s="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P008</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
           <t>1881-09-26</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>palacio</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>palacio</t>
+          <t>澳门：总督府</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>澳门：总督府</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
           <t>澳门</t>
         </is>
       </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="H4" s="2" t="n">
+        <v>22.19</v>
+      </c>
       <c r="I4" s="2" t="n">
-        <v>22.19</v>
-      </c>
-      <c r="J4" s="2" t="n">
         <v>113.538056</v>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>city-level</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>city-level</t>
+          <t>行政建筑</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>行政建筑</t>
+          <t>...el público le saluda con cohetes y petardos, que se confunden con los acordes de la música que graciosamente y en honor del pueblo chino, ha dispuesto el señor gobernador de la colonia que toque a su paso por delante del palacio.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>...el público le saluda con cohetes y petardos, que se confunden con los acordes de la música que graciosamente y en honor del pueblo chino, ha dispuesto el señor gobernador de la colonia que toque a su paso por delante del palacio.</t>
+          <t>……公众用火箭和鞭炮向它致敬，这些声音与音乐声交织在一起；为了向中国人民表示敬意，殖民地总督先生已安排音乐在龙经过总督府前时演奏。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>……公众用火箭和鞭炮向它致敬，这些声音与音乐声交织在一起；为了向中国人民表示敬意，殖民地总督先生已安排音乐在龙经过总督府前时演奏。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1442,12 +1427,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q4" s="0" t="inlineStr">
+      <c r="P4" s="0" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Special:EntityData/Q14773.json</t>
         </is>
@@ -1456,20 +1436,20 @@
     <row r="5" ht="170" customHeight="1" s="9">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P011</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
           <t>1882-12-08</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>11</v>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Hong-Kong</t>
+        </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Hong-Kong</t>
+          <t>香港</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1477,45 +1457,45 @@
           <t>香港</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>香港</t>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="H5" s="2" t="n">
+        <v>22.278333</v>
+      </c>
       <c r="I5" s="2" t="n">
-        <v>22.278333</v>
-      </c>
-      <c r="J5" s="2" t="n">
         <v>114.158611</v>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>city-level</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>city-level</t>
+          <t>城市</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>城市</t>
+          <t>Las noventa y tantas millas que separan al emporio chino de la colonia de Hong-Kong, y de las cuales más de dos tercios son de navegación fluvial, se recorren en unas siete horas en vapores de río...</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Las noventa y tantas millas que separan al emporio chino de la colonia de Hong-Kong, y de las cuales más de dos tercios son de navegación fluvial, se recorren en unas siete horas en vapores de río...</t>
+          <t>将中国商业中心与香港殖民地分隔开来的九十多英里路程，其中三分之二以上是内河航行，乘坐内河蒸汽船大约需要七个小时……</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>将中国商业中心与香港殖民地分隔开来的九十多英里路程，其中三分之二以上是内河航行，乘坐内河蒸汽船大约需要七个小时……</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -1523,12 +1503,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q5" s="0" t="inlineStr">
+      <c r="P5" s="0" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Special:EntityData/Q8646.json</t>
         </is>
@@ -1537,66 +1512,66 @@
     <row r="6" ht="102" customHeight="1" s="9">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P012</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
           <t>1882-12-08</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>12</v>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Boca Tigris</t>
+        </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Boca Tigris</t>
+          <t>虎门</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>虎门</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
           <t>东莞</t>
         </is>
       </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
           <t>area</t>
         </is>
       </c>
+      <c r="H6" s="2" t="n">
+        <v>22.816245</v>
+      </c>
       <c r="I6" s="2" t="n">
-        <v>22.816245</v>
-      </c>
-      <c r="J6" s="2" t="n">
         <v>113.6684225</v>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>区</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>区</t>
+          <t>Para Boca Tigris, fortificación que defiende la entrada del rio, es la primera sonrisa del excursionista...</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Para Boca Tigris, fortificación que defiende la entrada del rio, es la primera sonrisa del excursionista...</t>
+          <t>对于虎门——守卫河流入口的堡垒——这是旅行者的第一个微笑……</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>对于虎门——守卫河流入口的堡垒——这是旅行者的第一个微笑……</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1604,12 +1579,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q6" s="0" t="inlineStr">
+      <c r="P6" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=R5664991&amp;format=jsonv2</t>
         </is>
@@ -1618,66 +1588,66 @@
     <row r="7" ht="119" customHeight="1" s="9">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>P013</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
           <t>1882-12-08</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>13</v>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Wampoa</t>
+        </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Wampoa</t>
+          <t>黄埔</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>黄埔</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
           <t>area</t>
         </is>
       </c>
+      <c r="H7" s="2" t="n">
+        <v>23.1829382</v>
+      </c>
       <c r="I7" s="2" t="n">
-        <v>23.1829382</v>
-      </c>
-      <c r="J7" s="2" t="n">
         <v>113.47493</v>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>区</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>区</t>
+          <t>Remontando aquellas riberas amenizadas con las típicas torres de cinco, seis o siete pisos... llégase a Wampoa, avanzada de Cantón...</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Remontando aquellas riberas amenizadas con las típicas torres de cinco, seis o siete pisos... llégase a Wampoa, avanzada de Cantón...</t>
+          <t>沿着那些被典型的五、六、七层塔楼点缀的河岸上行……就到达了黄埔，广州的前哨……</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>沿着那些被典型的五、六、七层塔楼点缀的河岸上行……就到达了黄埔，广州的前哨……</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1685,12 +1655,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q7" s="0" t="inlineStr">
+      <c r="P7" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=R3987437&amp;format=jsonv2</t>
         </is>
@@ -1699,66 +1664,66 @@
     <row r="8" ht="51" customHeight="1" s="9">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P014</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
           <t>1882-12-08</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>14</v>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>emporio chino</t>
+        </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>emporio chino</t>
+          <t>广州城</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>广州城</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>overview</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>overview</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
           <t>city</t>
         </is>
       </c>
+      <c r="H8" s="2" t="n">
+        <v>23.13</v>
+      </c>
       <c r="I8" s="2" t="n">
-        <v>23.13</v>
-      </c>
-      <c r="J8" s="2" t="n">
         <v>113.26</v>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>city-level</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>city-level</t>
+          <t>城市</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>城市</t>
+          <t>Por fin se atraca: estamos en el emporio chino.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Por fin se atraca: estamos en el emporio chino.</t>
+          <t>终于靠岸了：我们到了中国商业中心。</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>终于靠岸了：我们到了中国商业中心。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1766,12 +1731,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q8" s="0" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Special:EntityData/Q16572.json</t>
         </is>
@@ -1780,66 +1740,66 @@
     <row r="9" ht="170" customHeight="1" s="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>P016</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
           <t>1882-12-08</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>16</v>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Shameen</t>
+        </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Shameen</t>
+          <t>沙面</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>沙面</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
           <t>area</t>
         </is>
       </c>
+      <c r="H9" s="2" t="n">
+        <v>23.1094481</v>
+      </c>
       <c r="I9" s="2" t="n">
-        <v>23.1094481</v>
-      </c>
-      <c r="J9" s="2" t="n">
         <v>113.2393051</v>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>岛屿</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>岛屿</t>
+          <t>Atravesando el puente de los señores... nos encontramos en Shameen; islote más grande que una manta de cama pequeña de matrimonio, cuyo terreno constituye la concesión o morada europea.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Atravesando el puente de los señores... nos encontramos en Shameen; islote más grande que una manta de cama pequeña de matrimonio, cuyo terreno constituye la concesión o morada europea.</t>
+          <t>穿过绅士桥……我们就到了沙面；这个小岛比一张小双人床的床单大不了多少，其土地构成了欧洲租界或居留地。</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>穿过绅士桥……我们就到了沙面；这个小岛比一张小双人床的床单大不了多少，其土地构成了欧洲租界或居留地。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1847,12 +1807,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q9" s="0" t="inlineStr">
+      <c r="P9" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=R6679655&amp;format=jsonv2</t>
         </is>
@@ -1861,66 +1816,66 @@
     <row r="10" ht="170" customHeight="1" s="9">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P022</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>22</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>La de los Quinientos ídolos</t>
+        </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>La de los Quinientos ídolos</t>
+          <t>华林寺/五百罗汉堂</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>华林寺/五百罗汉堂</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H10" s="2" t="n">
+        <v>23.1186158</v>
+      </c>
       <c r="I10" s="2" t="n">
-        <v>23.1186158</v>
-      </c>
-      <c r="J10" s="2" t="n">
         <v>113.241264</v>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>宗教建筑</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>宗教建筑</t>
+          <t>Las pagodas... Cuéntanse a centenares, por lo que no nos detendremos mas que en las que ofrezcan alguna particularidad. La de los Quinientos ídolos（广州华林寺） es sencillamente un museo de escultura...</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Las pagodas... Cuéntanse a centenares, por lo que no nos detendremos mas que en las que ofrezcan alguna particularidad. La de los Quinientos ídolos（广州华林寺） es sencillamente un museo de escultura...</t>
+          <t>寺庙……数以百计，因此我们只停留在那些有某种特色的寺庙。五百罗汉堂简直是一座雕塑博物馆……</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>寺庙……数以百计，因此我们只停留在那些有某种特色的寺庙。五百罗汉堂简直是一座雕塑博物馆……</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1928,12 +1883,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q10" s="0" t="inlineStr">
+      <c r="P10" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=W431484001&amp;format=jsonv2</t>
         </is>
@@ -1942,66 +1892,66 @@
     <row r="11" ht="102" customHeight="1" s="9">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P023</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>23</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>La de la Campana</t>
+        </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>La de la Campana</t>
+          <t>五仙观／岭南第一楼</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>五仙观／岭南第一楼</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H11" s="2" t="n">
+        <v>23.1233478</v>
+      </c>
       <c r="I11" s="2" t="n">
-        <v>23.1233478</v>
-      </c>
-      <c r="J11" s="2" t="n">
         <v>113.2544361</v>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>宗教建筑</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>宗教建筑</t>
+          <t>La de la Campana es sólo notable por el gigantesco tamaño de la que pende de una oscura y medio derruida linterna.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>La de la Campana es sólo notable por el gigantesco tamaño de la que pende de una oscura y medio derruida linterna.</t>
+          <t>钟寺之所以出名，仅仅是因为悬挂在一座昏暗且半毁的塔楼中的那口巨钟。</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>钟寺之所以出名，仅仅是因为悬挂在一座昏暗且半毁的塔楼中的那口巨钟。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2009,12 +1959,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q11" s="0" t="inlineStr">
+      <c r="P11" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=W363576776&amp;format=jsonv2</t>
         </is>
@@ -2023,66 +1968,66 @@
     <row r="12" ht="119" customHeight="1" s="9">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P025</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>25</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>La Pagoda de los Cerdos</t>
+        </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>La Pagoda de los Cerdos</t>
+          <t>海幢寺</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>海幢寺</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H12" s="2" t="n">
+        <v>23.1079575</v>
+      </c>
       <c r="I12" s="2" t="n">
-        <v>23.1079575</v>
-      </c>
-      <c r="J12" s="2" t="n">
         <v>113.2538565</v>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>宗教建筑</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>宗教建筑</t>
+          <t>La Pagoda de los Cerdos, así llamada por una pocilga en la que pasan feliz existencia cinco o seis ejemplares sagrados de ellos...</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>La Pagoda de los Cerdos, así llamada por una pocilga en la que pasan feliz existencia cinco o seis ejemplares sagrados de ellos...</t>
+          <t>猪庙，因一个猪圈而得名，里面五六头神圣的猪过着幸福的生活……</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>猪庙，因一个猪圈而得名，里面五六头神圣的猪过着幸福的生活……</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -2090,12 +2035,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q12" s="0" t="inlineStr">
+      <c r="P12" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=W363853167&amp;format=jsonv2</t>
         </is>
@@ -2104,66 +2044,66 @@
     <row r="13" ht="119" customHeight="1" s="9">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>P026</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>26</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>La de los Cinco pisos</t>
+        </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>La de los Cinco pisos</t>
+          <t>镇海楼</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>镇海楼</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H13" s="2" t="n">
+        <v>23.1406034</v>
+      </c>
       <c r="I13" s="2" t="n">
-        <v>23.1406034</v>
-      </c>
-      <c r="J13" s="2" t="n">
         <v>113.2602757</v>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>行政建筑</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>行政建筑</t>
+          <t>La de los Cinco pisos, desmantelada, no sirve ya mas que de mirador, en gracia de su altura, y fue cuartel general del ejército de ocupación.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>La de los Cinco pisos, desmantelada, no sirve ya mas que de mirador, en gracia de su altura, y fue cuartel general del ejército de ocupación.</t>
+          <t>五层塔，已被废弃，仅因其高度而用作观景台，曾是占领军的总部。</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>五层塔，已被废弃，仅因其高度而用作观景台，曾是占领军的总部。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -2171,12 +2111,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q13" s="0" t="inlineStr">
+      <c r="P13" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=W146688561&amp;format=jsonv2</t>
         </is>
@@ -2185,66 +2120,66 @@
     <row r="14" ht="153" customHeight="1" s="9">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>P028</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>28</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>la Catedral erigida en el centro del barrio tártaro</t>
+        </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>la Catedral erigida en el centro del barrio tártaro</t>
+          <t>广州圣心大教堂</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>广州圣心大教堂</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H14" s="2" t="n">
+        <v>23.1173975</v>
+      </c>
       <c r="I14" s="2" t="n">
-        <v>23.1173975</v>
-      </c>
-      <c r="J14" s="2" t="n">
         <v>113.2547256</v>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>宗教建筑</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>宗教建筑</t>
+          <t>Cerremos esta crónica religiosa con cuatro palabras sobre la Catedral erigida en el centro del barrio tártaro. De orden gótico, está tallada en duro granito y recuerda la de Amiens.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Cerremos esta crónica religiosa con cuatro palabras sobre la Catedral erigida en el centro del barrio tártaro. De orden gótico, está tallada en duro granito y recuerda la de Amiens.</t>
+          <t>让我们用几句话来结束这篇宗教纪事，谈谈建在鞑靼区中心的教堂。它属于哥特式，用坚硬的花岗岩雕成，让人想起亚眠大教堂。</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>让我们用几句话来结束这篇宗教纪事，谈谈建在鞑靼区中心的教堂。它属于哥特式，用坚硬的花岗岩雕成，让人想起亚眠大教堂。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -2252,12 +2187,7 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q14" s="0" t="inlineStr">
+      <c r="P14" s="0" t="inlineStr">
         <is>
           <t>https://nominatim.openstreetmap.org/lookup?osm_ids=W542890833&amp;format=jsonv2</t>
         </is>
@@ -2266,66 +2196,66 @@
     <row r="15" ht="85" customHeight="1" s="9">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P031</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>31</v>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>el yamen del gobernador</t>
+        </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>el yamen del gobernador</t>
+          <t>两广总督衙门旧址（今广东省民政厅）</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>两广总督衙门旧址（今广东省民政厅）</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
           <t>广州</t>
         </is>
       </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
           <t>site</t>
         </is>
       </c>
+      <c r="H15" s="2" t="n">
+        <v>23.13196</v>
+      </c>
       <c r="I15" s="2" t="n">
-        <v>23.13196</v>
-      </c>
-      <c r="J15" s="2" t="n">
         <v>113.26091</v>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>行政建筑</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>行政建筑</t>
+          <t>Esto me da pie para relatar nuestra visita al yamen o palacio del feudal lugarteniente del emperador.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Esto me da pie para relatar nuestra visita al yamen o palacio del feudal lugarteniente del emperador.</t>
+          <t>这让我有机会讲述我们拜访皇帝封建副手——即总督——的衙门或宫殿的经过。</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>这让我有机会讲述我们拜访皇帝封建副手——即总督——的衙门或宫殿的经过。</t>
+          <t>null</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2333,19 +2263,14 @@
           <t>null</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
+      <c r="P15" s="0" t="inlineStr">
         <is>
           <t>https://www.yuexiu.gov.cn/data/cms/category/xzzfsj/kejj1548668945490809.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q15"/>
+  <autoFilter ref="A1:P15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>